<commit_message>
fix: delivery order bugs
- harga manual itu bisa naik tapi gabisa turun.
</commit_message>
<xml_diff>
--- a/test/delivery-order-flow.xlsx
+++ b/test/delivery-order-flow.xlsx
@@ -871,7 +871,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">POST /delivery-order/store: item1 use_manual_price=false, item2 manual=katalog-500; detail CUSTOMER_PO_NUMBER/CASHBACK_PPH_4/BIAYA_BONGKAR/PAYMENT_TERMS</t>
+          <t xml:space="preserve">POST /delivery-order/store: item1 use_manual_price=false, item2 manual=katalog+500; detail CUSTOMER_PO_NUMBER/CASHBACK_PPH_4/BIAYA_BONGKAR/PAYMENT_TERMS</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -881,7 +881,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">details: nomor_po_pelanggan=PO-REV-001, cashback_pph_4=150000, biaya_bongkar=75000, syarat_pembayaran="Invoice, Faktur Pajak, Kwitansi", manual_price=true; item p22 base manual 13360; grand=116205 = 76125+40080 (tanpa potongan field opsional)</t>
+          <t xml:space="preserve">details: nomor_po_pelanggan=PO-REV-001, cashback_pph_4=150000, biaya_bongkar=75000, syarat_pembayaran="Invoice, Faktur Pajak, Kwitansi", manual_price=true; item p22 unit manual 15680 (=15180+500) total=47040; grand=115825.65 = 68785.65+47040 (tanpa potongan field opsional)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -898,22 +898,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Revisi 3: cap harga manual (server)</t>
+          <t xml:space="preserve">Revisi 3: lantai harga manual (server, buat dokumen)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">POST /delivery-order/store use_manual_price=true unit_price=katalog+1</t>
+          <t xml:space="preserve">POST /delivery-order/store use_manual_price=true unit_price=katalog (sama persis) | katalog-1 | katalog+500</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ditolak (error form), tidak ada dokumen tersimpan</t>
+          <t xml:space="preserve">unit_price &gt;= harga daftar diterima; unit_price &lt; harga daftar ditolak (error form) dan tidak ada dokumen baru</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">302 -&gt; /delivery-order/create; jumlah dokumen sebelum=1 sesudah=1; pesan "melebihi harga daftar" dihitung DeliveryOrderCalculator::manualPrice()</t>
+          <t xml:space="preserve">katalog 15180: =15180 -&gt; 302 documents total=45540 (tx 917); =15179 -&gt; 302 kembali ke /delivery-order/create, jumlah DO tidak bertambah, errors.delivery_order = "Harga manual ... di bawah harga daftar (minimal Rp15.180,00)"; =15680 -&gt; 302 documents total=47040 (tx 918). Pesan dihitung DeliveryOrderCalculator::manualPrice()</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1205,6 +1205,390 @@
         </is>
       </c>
       <c r="F36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Build frontend (Revisi DO)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">npm run build</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Build sukses; chunk halaman daftar revisi ter-generate</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IndexRevisions-BhNqvKiV.js ter-generate di samping IndexRevisions PO (W_grFGuH.js)</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">37</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Route revisi</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">php artisan route:list --path=delivery-order</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 route revisi terdaftar: daftar, form, submit</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">delivery-order.revisions (GET /revisions), delivery-order.revise (GET /{id}/revise), delivery-order.revise.update (PUT /{id}/revise)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">38</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Daftar revisi</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /delivery-order/revisions</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">200 komponen DeliveryOrder/IndexRevisions; hanya NEED_REVISION; membawa created_by untuk guard</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">total=1, status=NEED_REVISION, created_by=1, alasan revisi ikut tampil</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">39</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Guard halaman revisi</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /delivery-order/revisions + /{id}/revise sebagai user sales lain (2 user)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">403, bukan halaman revisi</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET revisi -&gt; 403 pada kedua user non-pembuat</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prefill form revisi</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /delivery-order/{id}/revise (props deliveryOrder -&gt; useDeliveryOrder mode=revise)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Form ter-hydrate dari dokumen: nomor DO tidak berubah, tanggal/PO/cashback/bongkar/termin/PPN/flag manual terisi, item &amp; snapshot promo terbawa</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">do_number=DO-2610-000001, delivery_date=2026-10-11, nomor_po_pelanggan=PO-REV-001, cashback=150000, biaya_bongkar=75000, syarat="Invoice, Faktur Pajak, Kwitansi", items=2, promo=true unit_price_before=16675 (= harga daftar, sumber hydrate), unit_price=13757.13 (hasil diskon), use_manual_price terbawa, ppn=true</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">41</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Submit revisi</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PUT /delivery-order/{id}/revise (qty 7 &amp; 4, tanggal 2026-10-13, PO-REV-002, harga manual katalog+700, document_code sengaja dikirim salah)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">302 ke halaman detail; document_code diabaikan; nominal dihitung ulang server; approval dibuat ulang; stok dialokasikan ulang; keputusan lama diarsipkan</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">document_code tetap DO-2610-000001; desc/tgl/PO berubah; total p22 = 63520 (=15880*4, 15180+700); sub=143981.91 tax=15838.00 grand=159819.91 disc=20425.09 (grand = jumlah total_price item; sub+PPN=grand); rantai baru 5 langkah semua PENDING, langkah 1 Sales/Sales Manager, BD tetap ada (harga manual); arsip=5 berisi NEED_REVISION; journals OUT 21=7 &amp; 22=4 tanpa baris ganda</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">42</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Revisi saat masih PENDING ditolak</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PUT /delivery-order/{id}/revise setelah dokumen kembali PENDING</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">302 kembali (bukan 500); isi dokumen, approval, arsip tidak berubah</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">desc tetap "Revisi: qty &amp; tanggal diganti", qty=7, approvals=5, arsip=5</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">43</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gagal revisi: stok kurang</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PUT /delivery-order/{id}/revise quantity=999999</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bukan 500; kembali ke form revisi; dokumen &amp; stok tidak berubah</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">302 ke /delivery-order/{id}/revise; desc/qty tetap (4), rantai &amp; arsip utuh, journals OUT 7 &amp; 4 tidak berubah</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">44</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CSRF token revisi</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PUT /delivery-order/{id}/revise tanpa header X-XSRF-TOKEN (cookie session sah)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ditolak 419, dokumen tidak berubah</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">code=419 (halaman error CSRF); description tetap "Revisi: qty &amp; tanggal diganti"</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">45</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pembersihan data uji (putaran Revisi DO)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hapus DO uji 919 + baris terkait</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sisa 0 DO, saldo stok kembali</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO tersisa 0; balance p21=150, p22=100, p23=120</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">46</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lantai harga manual di form revisi</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PUT /delivery-order/{id}/revise dengan unit_price manual = harga daftar - 1 (payload dokumen NEED_REVISION)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ditolak (302 kembali ke form revisi, bukan 500); dokumen, qty, rantai approval, arsip tidak berubah; pesan tampil di form</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">code=302 -&gt; /delivery-order/{id}/revise; desc &amp; qty tetap; total p22 tetap 63520; approvals=5, arsip=5; errors.delivery_order = "Harga manual untuk produk \"Tepung Terigu Protein Sedang\" di bawah harga daftar (minimal Rp15.180,00)." (77 pass, 0 fail)</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">47</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Frontend: lantai harga manual</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">npm run build + resources/js (ProductInput.vue, useDeliveryOrder.ts)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Input manual memakai :min = harga daftar (tanpa :max), hint "Minimal ...", dan draftError memblokir harga di bawah daftar dengan pesan serupa server</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">build sukses 28.71s; NInputNumber :min="useManual ? priceFloor : 0" (priceCap -&gt; priceFloor); hint "Minimal Rp15.180 — tidak boleh turun dari harga daftar."; draftError: unit_price &lt; product.price -&gt; "di bawah harga daftar (minimal ...)"</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
         <is>
           <t xml:space="preserve">PASS</t>
         </is>

</xml_diff>